<commit_message>
rerun everything from empty and get the same answers, reassuringly
</commit_message>
<xml_diff>
--- a/04_Figures/S5/c_data/S5.xlsx
+++ b/04_Figures/S5/c_data/S5.xlsx
@@ -1846,7 +1846,7 @@
     <t>01_Processing/07_Module_Characterisation/c_data/module_characterisation.xlsx</t>
   </si>
   <si>
-    <t>5e561cc796eef082629205d0768131b9</t>
+    <t>94cadc901960bff29e73192652852642</t>
   </si>
   <si>
     <t>modules</t>
@@ -1864,7 +1864,7 @@
     <t>01_Processing/06_Module_Building/c_data/module_building.xlsx</t>
   </si>
   <si>
-    <t>df4d5af4fd36983481be113e72db4d4d</t>
+    <t>eeacbc52b19a3a95fb620dd873a2b3d7</t>
   </si>
   <si>
     <t>BiocManager</t>

</xml_diff>

<commit_message>
let F4 pick its pathways the way F3 does, with one tree to rule them both
</commit_message>
<xml_diff>
--- a/04_Figures/S5/c_data/S5.xlsx
+++ b/04_Figures/S5/c_data/S5.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2845" uniqueCount="727">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2854" uniqueCount="733">
   <si>
     <t>sheet</t>
   </si>
@@ -1963,6 +1963,15 @@
     <t>0.9.8</t>
   </si>
   <si>
+    <t>ggtext</t>
+  </si>
+  <si>
+    <t>0.2.0</t>
+  </si>
+  <si>
+    <t>CRAN (R 4.6.1)</t>
+  </si>
+  <si>
     <t>glue</t>
   </si>
   <si>
@@ -1975,15 +1984,18 @@
     <t>1.2.5</t>
   </si>
   <si>
-    <t>CRAN (R 4.6.1)</t>
-  </si>
-  <si>
     <t>gridExtra</t>
   </si>
   <si>
     <t>2.3</t>
   </si>
   <si>
+    <t>gridtext</t>
+  </si>
+  <si>
+    <t>0.1.6</t>
+  </si>
+  <si>
     <t>gtable</t>
   </si>
   <si>
@@ -2195,6 +2207,12 @@
   </si>
   <si>
     <t>3.0.2</t>
+  </si>
+  <si>
+    <t>xml2</t>
+  </si>
+  <si>
+    <t>1.5.2</t>
   </si>
   <si>
     <t>yaml</t>
@@ -16272,7 +16290,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -16470,18 +16488,18 @@
         <v>648</v>
       </c>
       <c r="C18" t="s">
-        <v>617</v>
+        <v>649</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B19" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="C19" t="s">
-        <v>651</v>
+        <v>617</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -16492,7 +16510,7 @@
         <v>653</v>
       </c>
       <c r="C20" t="s">
-        <v>617</v>
+        <v>649</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -16536,7 +16554,7 @@
         <v>661</v>
       </c>
       <c r="C24" t="s">
-        <v>651</v>
+        <v>617</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -16558,7 +16576,7 @@
         <v>665</v>
       </c>
       <c r="C26" t="s">
-        <v>617</v>
+        <v>649</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -16723,7 +16741,7 @@
         <v>695</v>
       </c>
       <c r="C41" t="s">
-        <v>651</v>
+        <v>617</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -16745,7 +16763,7 @@
         <v>699</v>
       </c>
       <c r="C43" t="s">
-        <v>617</v>
+        <v>649</v>
       </c>
     </row>
     <row r="44" spans="1:3">
@@ -16819,7 +16837,7 @@
         <v>712</v>
       </c>
       <c r="B50" t="s">
-        <v>673</v>
+        <v>713</v>
       </c>
       <c r="C50" t="s">
         <v>617</v>
@@ -16827,10 +16845,10 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B51" t="s">
-        <v>630</v>
+        <v>715</v>
       </c>
       <c r="C51" t="s">
         <v>617</v>
@@ -16838,7 +16856,7 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="B52" t="s">
         <v>677</v>
@@ -16849,10 +16867,10 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="B53" t="s">
-        <v>638</v>
+        <v>630</v>
       </c>
       <c r="C53" t="s">
         <v>617</v>
@@ -16860,10 +16878,10 @@
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="B54" t="s">
-        <v>717</v>
+        <v>681</v>
       </c>
       <c r="C54" t="s">
         <v>617</v>
@@ -16871,10 +16889,10 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B55" t="s">
-        <v>719</v>
+        <v>638</v>
       </c>
       <c r="C55" t="s">
         <v>617</v>
@@ -16885,7 +16903,7 @@
         <v>720</v>
       </c>
       <c r="B56" t="s">
-        <v>663</v>
+        <v>721</v>
       </c>
       <c r="C56" t="s">
         <v>617</v>
@@ -16893,10 +16911,10 @@
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B57" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="C57" t="s">
         <v>617</v>
@@ -16904,10 +16922,10 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B58" t="s">
-        <v>724</v>
+        <v>667</v>
       </c>
       <c r="C58" t="s">
         <v>617</v>
@@ -16921,6 +16939,39 @@
         <v>726</v>
       </c>
       <c r="C59" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" t="s">
+        <v>727</v>
+      </c>
+      <c r="B60" t="s">
+        <v>728</v>
+      </c>
+      <c r="C60" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" t="s">
+        <v>729</v>
+      </c>
+      <c r="B61" t="s">
+        <v>730</v>
+      </c>
+      <c r="C61" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" t="s">
+        <v>731</v>
+      </c>
+      <c r="B62" t="s">
+        <v>732</v>
+      </c>
+      <c r="C62" t="s">
         <v>617</v>
       </c>
     </row>

</xml_diff>

<commit_message>
read S5's soft power from the step instead of trusting a twelve typed by hand
</commit_message>
<xml_diff>
--- a/04_Figures/S5/c_data/S5.xlsx
+++ b/04_Figures/S5/c_data/S5.xlsx
@@ -37,7 +37,7 @@
     <t>a_characterisation</t>
   </si>
   <si>
-    <t>Panel a: top three ORA sets per module (part ora) and the ten highest-kME members with their grid position (part member).</t>
+    <t>Panel a: top 3 ORA sets per module (part ora) and the 10 highest-kME members with their grid position (part member).</t>
   </si>
   <si>
     <t>b_string</t>
@@ -49,7 +49,7 @@
     <t>c_module_qc</t>
   </si>
   <si>
-    <t>Panel c: modules and grey proteins per soft power (part network) and each power-12 module's kept share at powers 10, 14 and 19 (part kept_share).</t>
+    <t>Panel c: modules and grey proteins per soft power (part network) and each power-12 module's kept share at powers 10, 14, 19 (part kept_share).</t>
   </si>
   <si>
     <t>input_manifest</t>

</xml_diff>